<commit_message>
Excel upload feature was realized
</commit_message>
<xml_diff>
--- a/Catalog_Testovoe.xlsx
+++ b/Catalog_Testovoe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PyCharm\DjangoRESTTest\myProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\work\Python\Projects\django\testproject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB91CD49-BC5E-44CF-B408-A5BE31753492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B119ED-9ED2-4188-9DE3-260B6BEF930C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="900" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -405,17 +405,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -435,7 +435,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1000</v>
       </c>
@@ -447,7 +447,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1001</v>
       </c>
@@ -461,7 +461,7 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1002</v>
       </c>
@@ -481,7 +481,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1003</v>
       </c>
@@ -501,7 +501,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>1003</v>
       </c>
@@ -521,7 +521,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>1004</v>
       </c>
@@ -535,7 +535,7 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1005</v>
       </c>
@@ -555,7 +555,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>1006</v>
       </c>
@@ -575,7 +575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>

</xml_diff>